<commit_message>
Gerando certificados em massa (RPA)
</commit_message>
<xml_diff>
--- a/Word/Alunos.xlsx
+++ b/Word/Alunos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23801"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Curso Lógica de Programação\Python\Word\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\eric.psouza\Documents\Cursos\Curso Lógica de Programação (Python)\Word\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E16C0048-EB67-4B4B-81A5-288382A387DF}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B9371B-ABFC-4237-89EE-68DD3F9207EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{BAEC095C-CF3A-4E6D-8D9A-83FDFC985053}"/>
+    <workbookView xWindow="-21720" yWindow="645" windowWidth="21840" windowHeight="13740" xr2:uid="{BAEC095C-CF3A-4E6D-8D9A-83FDFC985053}"/>
   </bookViews>
   <sheets>
     <sheet name="Nomes" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Aluno</t>
   </si>
@@ -40,6 +40,9 @@
   </si>
   <si>
     <t>Claudia Ferreira de Souza</t>
+  </si>
+  <si>
+    <t>Teste Aluno Extra</t>
   </si>
 </sst>
 </file>
@@ -76,7 +79,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -99,14 +102,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -125,9 +140,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -165,7 +180,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -271,7 +286,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -413,7 +428,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -421,7 +436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0A1AA0A-25C7-4052-8642-6C123477577B}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="63.5546875" customWidth="1"/>
@@ -452,6 +467,11 @@
         <v>4</v>
       </c>
     </row>
+    <row r="6" spans="1:1" ht="33.6" x14ac:dyDescent="0.65">
+      <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>

</xml_diff>